<commit_message>
Capture npm dev refresh outputs
</commit_message>
<xml_diff>
--- a/output/Nasarawa/results.xlsx
+++ b/output/Nasarawa/results.xlsx
@@ -20664,7 +20664,11 @@
         <v>86117</v>
       </c>
       <c r="M132" t="inlineStr"/>
-      <c r="N132" t="inlineStr"/>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>1781985243008</t>
+        </is>
+      </c>
       <c r="O132" t="n">
         <v>0</v>
       </c>
@@ -20685,7 +20689,11 @@
         <v>0</v>
       </c>
       <c r="V132" t="inlineStr"/>
-      <c r="W132" t="inlineStr"/>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2987/26/526/6008/85053/f14edfb4-9d79-4b46-a80d-bac4d2ff237f.jpg</t>
+        </is>
+      </c>
       <c r="X132" t="n">
         <v>0</v>
       </c>
@@ -41175,7 +41183,11 @@
         <v>162671</v>
       </c>
       <c r="M267" t="inlineStr"/>
-      <c r="N267" t="inlineStr"/>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>1781985422478</t>
+        </is>
+      </c>
       <c r="O267" t="n">
         <v>0</v>
       </c>
@@ -41196,7 +41208,11 @@
         <v>0</v>
       </c>
       <c r="V267" t="inlineStr"/>
-      <c r="W267" t="inlineStr"/>
+      <c r="W267" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2987/26/534/6114/657913/4ee608dd-fbc3-4130-941c-4a86fc3c2b4b.jpg</t>
+        </is>
+      </c>
       <c r="X267" t="n">
         <v>0</v>
       </c>
@@ -73515,7 +73531,11 @@
         <v>162917</v>
       </c>
       <c r="M481" t="inlineStr"/>
-      <c r="N481" t="inlineStr"/>
+      <c r="N481" t="inlineStr">
+        <is>
+          <t>1781984883117</t>
+        </is>
+      </c>
       <c r="O481" t="n">
         <v>0</v>
       </c>
@@ -73536,7 +73556,11 @@
         <v>0</v>
       </c>
       <c r="V481" t="inlineStr"/>
-      <c r="W481" t="inlineStr"/>
+      <c r="W481" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2987/26/536/6143/658207/eabfb1ad-f7d4-4f20-9893-3e9e87fa3d75.jpg</t>
+        </is>
+      </c>
       <c r="X481" t="n">
         <v>0</v>
       </c>
@@ -90147,10 +90171,10 @@
         <v>14</v>
       </c>
       <c r="AG7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AH7" t="n">
-        <v>35.7</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="8">
@@ -91138,10 +91162,10 @@
         <v>16</v>
       </c>
       <c r="AG16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AH16" t="n">
-        <v>43.8</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -92458,10 +92482,10 @@
         <v>12</v>
       </c>
       <c r="AG28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH28" t="n">
-        <v>50</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="29">
@@ -93624,10 +93648,10 @@
         <v>206</v>
       </c>
       <c r="AF2" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AG2" t="n">
-        <v>50.5</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3">
@@ -93729,10 +93753,10 @@
         <v>255</v>
       </c>
       <c r="AF3" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AG3" t="n">
-        <v>25.9</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="4">
@@ -93834,10 +93858,10 @@
         <v>122</v>
       </c>
       <c r="AF4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AG4" t="n">
-        <v>40.2</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -94115,13 +94139,13 @@
         <v>583</v>
       </c>
       <c r="AE2" t="n">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AF2" t="n">
         <v>583</v>
       </c>
       <c r="AG2" t="n">
-        <v>37.6</v>
+        <v>38.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 15:09:47
</commit_message>
<xml_diff>
--- a/output/Nasarawa/results.xlsx
+++ b/output/Nasarawa/results.xlsx
@@ -93648,10 +93648,10 @@
         <v>206</v>
       </c>
       <c r="AF2" t="n">
-        <v>105</v>
+        <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -93753,10 +93753,10 @@
         <v>255</v>
       </c>
       <c r="AF3" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>26.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -93858,10 +93858,10 @@
         <v>122</v>
       </c>
       <c r="AF4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -94139,13 +94139,13 @@
         <v>583</v>
       </c>
       <c r="AE2" t="n">
-        <v>222</v>
+        <v>0</v>
       </c>
       <c r="AF2" t="n">
         <v>583</v>
       </c>
       <c r="AG2" t="n">
-        <v>38.1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 15:23:31
</commit_message>
<xml_diff>
--- a/output/Nasarawa/results.xlsx
+++ b/output/Nasarawa/results.xlsx
@@ -93648,10 +93648,10 @@
         <v>206</v>
       </c>
       <c r="AF2" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3">
@@ -93753,10 +93753,10 @@
         <v>255</v>
       </c>
       <c r="AF3" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="4">
@@ -93858,10 +93858,10 @@
         <v>122</v>
       </c>
       <c r="AF4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -94139,13 +94139,13 @@
         <v>583</v>
       </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>222</v>
       </c>
       <c r="AF2" t="n">
         <v>583</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>38.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>